<commit_message>
Update Labor Nonlabor Resources
</commit_message>
<xml_diff>
--- a/boq-resource-id-hrs.xlsx
+++ b/boq-resource-id-hrs.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TIA_Program\OCB_01\Temp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TIA_Program\OCB_01\resource assignment-python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B6054DF7-F7D6-4520-9D11-F2DED7ED216B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC28CB8B-3FC4-4920-877E-1D1E65DEBD82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{43D02350-C60B-49FE-B2F2-F8F6D5DA8777}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="889" uniqueCount="105">
   <si>
     <t>BOQ Item No.</t>
   </si>
@@ -279,6 +279,78 @@
   </si>
   <si>
     <t>iii</t>
+  </si>
+  <si>
+    <t>Resource Type</t>
+  </si>
+  <si>
+    <t>Nonlabor</t>
+  </si>
+  <si>
+    <t>SKILLED</t>
+  </si>
+  <si>
+    <t>Labor</t>
+  </si>
+  <si>
+    <t>3.2.1.3</t>
+  </si>
+  <si>
+    <t>3.2.1.4</t>
+  </si>
+  <si>
+    <t>UN-SKILLED</t>
+  </si>
+  <si>
+    <t>3.2.2.7</t>
+  </si>
+  <si>
+    <t>3.2.2.8</t>
+  </si>
+  <si>
+    <t>3.2.2.9</t>
+  </si>
+  <si>
+    <t>3.2.2.10</t>
+  </si>
+  <si>
+    <t>3.2.2.11</t>
+  </si>
+  <si>
+    <t>3.2.2.14</t>
+  </si>
+  <si>
+    <t>3.2.2.15c</t>
+  </si>
+  <si>
+    <t>3.2.3.6b</t>
+  </si>
+  <si>
+    <t>3.2.12.6</t>
+  </si>
+  <si>
+    <t>3.2.12.6b</t>
+  </si>
+  <si>
+    <t>3.2.12.6d</t>
+  </si>
+  <si>
+    <t>3.2.12.7</t>
+  </si>
+  <si>
+    <t>3.2.12.7d</t>
+  </si>
+  <si>
+    <t>3.2.12.7e</t>
+  </si>
+  <si>
+    <t>v</t>
+  </si>
+  <si>
+    <t>Skilled Labor</t>
+  </si>
+  <si>
+    <t>Unskilled Labor</t>
   </si>
 </sst>
 </file>
@@ -650,10 +722,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCD7A653-10A5-4B3D-B832-9CDBCFD428FB}">
-  <dimension ref="A1:D119"/>
+  <dimension ref="A1:E222"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="3" width="18.375" customWidth="1"/>
+    <col min="4" max="4" width="17.25" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -661,13 +737,16 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -675,13 +754,16 @@
         <v>5</v>
       </c>
       <c r="C2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D2" t="s">
         <v>6</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -689,13 +771,16 @@
         <v>7</v>
       </c>
       <c r="C3" t="s">
+        <v>82</v>
+      </c>
+      <c r="D3" t="s">
         <v>8</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>4.3999999999999997E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -703,13 +788,16 @@
         <v>5</v>
       </c>
       <c r="C4" t="s">
+        <v>82</v>
+      </c>
+      <c r="D4" t="s">
         <v>6</v>
       </c>
-      <c r="D4">
+      <c r="E4">
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -717,13 +805,16 @@
         <v>7</v>
       </c>
       <c r="C5" t="s">
+        <v>82</v>
+      </c>
+      <c r="D5" t="s">
         <v>8</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>4.3999999999999997E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -731,13 +822,16 @@
         <v>5</v>
       </c>
       <c r="C6" t="s">
+        <v>82</v>
+      </c>
+      <c r="D6" t="s">
         <v>6</v>
       </c>
-      <c r="D6">
+      <c r="E6">
         <v>0.02</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -745,13 +839,16 @@
         <v>11</v>
       </c>
       <c r="C7" t="s">
+        <v>82</v>
+      </c>
+      <c r="D7" t="s">
         <v>12</v>
       </c>
-      <c r="D7">
+      <c r="E7">
         <v>0.01</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -759,13 +856,16 @@
         <v>13</v>
       </c>
       <c r="C8" t="s">
+        <v>82</v>
+      </c>
+      <c r="D8" t="s">
         <v>14</v>
       </c>
-      <c r="D8">
+      <c r="E8">
         <v>0.01</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -773,13 +873,16 @@
         <v>15</v>
       </c>
       <c r="C9" t="s">
+        <v>82</v>
+      </c>
+      <c r="D9" t="s">
         <v>16</v>
       </c>
-      <c r="D9">
+      <c r="E9">
         <v>0.02</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -787,13 +890,16 @@
         <v>7</v>
       </c>
       <c r="C10" t="s">
+        <v>82</v>
+      </c>
+      <c r="D10" t="s">
         <v>8</v>
       </c>
-      <c r="D10">
+      <c r="E10">
         <v>8.3333333333333329E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -801,13 +907,16 @@
         <v>17</v>
       </c>
       <c r="C11" t="s">
+        <v>82</v>
+      </c>
+      <c r="D11" t="s">
         <v>18</v>
       </c>
-      <c r="D11">
+      <c r="E11">
         <v>0.02</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -815,13 +924,16 @@
         <v>5</v>
       </c>
       <c r="C12" t="s">
+        <v>82</v>
+      </c>
+      <c r="D12" t="s">
         <v>6</v>
       </c>
-      <c r="D12">
+      <c r="E12">
         <v>0.02</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>19</v>
       </c>
@@ -829,13 +941,16 @@
         <v>11</v>
       </c>
       <c r="C13" t="s">
+        <v>82</v>
+      </c>
+      <c r="D13" t="s">
         <v>12</v>
       </c>
-      <c r="D13">
+      <c r="E13">
         <v>0.01</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>19</v>
       </c>
@@ -843,13 +958,16 @@
         <v>13</v>
       </c>
       <c r="C14" t="s">
+        <v>82</v>
+      </c>
+      <c r="D14" t="s">
         <v>14</v>
       </c>
-      <c r="D14">
+      <c r="E14">
         <v>0.01</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -857,13 +975,16 @@
         <v>15</v>
       </c>
       <c r="C15" t="s">
+        <v>82</v>
+      </c>
+      <c r="D15" t="s">
         <v>16</v>
       </c>
-      <c r="D15">
+      <c r="E15">
         <v>0.02</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -871,13 +992,16 @@
         <v>7</v>
       </c>
       <c r="C16" t="s">
+        <v>82</v>
+      </c>
+      <c r="D16" t="s">
         <v>8</v>
       </c>
-      <c r="D16">
+      <c r="E16">
         <v>8.3333333333333329E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>19</v>
       </c>
@@ -885,13 +1009,16 @@
         <v>17</v>
       </c>
       <c r="C17" t="s">
+        <v>82</v>
+      </c>
+      <c r="D17" t="s">
         <v>18</v>
       </c>
-      <c r="D17">
+      <c r="E17">
         <v>0.02</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -899,13 +1026,16 @@
         <v>13</v>
       </c>
       <c r="C18" t="s">
+        <v>82</v>
+      </c>
+      <c r="D18" t="s">
         <v>14</v>
       </c>
-      <c r="D18">
+      <c r="E18">
         <v>0.02</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>20</v>
       </c>
@@ -913,13 +1043,16 @@
         <v>15</v>
       </c>
       <c r="C19" t="s">
+        <v>82</v>
+      </c>
+      <c r="D19" t="s">
         <v>16</v>
       </c>
-      <c r="D19">
+      <c r="E19">
         <v>0.04</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>20</v>
       </c>
@@ -927,13 +1060,16 @@
         <v>21</v>
       </c>
       <c r="C20" t="s">
+        <v>82</v>
+      </c>
+      <c r="D20" t="s">
         <v>22</v>
       </c>
-      <c r="D20">
+      <c r="E20">
         <v>0.04</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -941,13 +1077,16 @@
         <v>7</v>
       </c>
       <c r="C21" t="s">
+        <v>82</v>
+      </c>
+      <c r="D21" t="s">
         <v>8</v>
       </c>
-      <c r="D21">
+      <c r="E21">
         <v>8.3333333333333329E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>20</v>
       </c>
@@ -955,13 +1094,16 @@
         <v>17</v>
       </c>
       <c r="C22" t="s">
+        <v>82</v>
+      </c>
+      <c r="D22" t="s">
         <v>18</v>
       </c>
-      <c r="D22">
+      <c r="E22">
         <v>3.3000000000000002E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>23</v>
       </c>
@@ -969,13 +1111,16 @@
         <v>24</v>
       </c>
       <c r="C23" t="s">
+        <v>82</v>
+      </c>
+      <c r="D23" t="s">
         <v>25</v>
       </c>
-      <c r="D23">
+      <c r="E23">
         <v>6.2827225130890049E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -983,13 +1128,16 @@
         <v>26</v>
       </c>
       <c r="C24" t="s">
+        <v>82</v>
+      </c>
+      <c r="D24" t="s">
         <v>27</v>
       </c>
-      <c r="D24">
+      <c r="E24">
         <v>6.2827225130890049E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -997,13 +1145,16 @@
         <v>28</v>
       </c>
       <c r="C25" t="s">
+        <v>82</v>
+      </c>
+      <c r="D25" t="s">
         <v>29</v>
       </c>
-      <c r="D25">
+      <c r="E25">
         <v>0.1256544502617801</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>23</v>
       </c>
@@ -1011,13 +1162,16 @@
         <v>7</v>
       </c>
       <c r="C26" t="s">
+        <v>82</v>
+      </c>
+      <c r="D26" t="s">
         <v>8</v>
       </c>
-      <c r="D26">
+      <c r="E26">
         <v>8.3333333333333329E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>30</v>
       </c>
@@ -1025,13 +1179,16 @@
         <v>24</v>
       </c>
       <c r="C27" t="s">
+        <v>82</v>
+      </c>
+      <c r="D27" t="s">
         <v>25</v>
       </c>
-      <c r="D27">
+      <c r="E27">
         <v>6.2827225130890049E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>30</v>
       </c>
@@ -1039,13 +1196,16 @@
         <v>26</v>
       </c>
       <c r="C28" t="s">
+        <v>82</v>
+      </c>
+      <c r="D28" t="s">
         <v>27</v>
       </c>
-      <c r="D28">
+      <c r="E28">
         <v>6.2827225130890049E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>30</v>
       </c>
@@ -1053,13 +1213,16 @@
         <v>28</v>
       </c>
       <c r="C29" t="s">
+        <v>82</v>
+      </c>
+      <c r="D29" t="s">
         <v>29</v>
       </c>
-      <c r="D29">
+      <c r="E29">
         <v>0.1256544502617801</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>30</v>
       </c>
@@ -1067,13 +1230,16 @@
         <v>7</v>
       </c>
       <c r="C30" t="s">
+        <v>82</v>
+      </c>
+      <c r="D30" t="s">
         <v>8</v>
       </c>
-      <c r="D30">
+      <c r="E30">
         <v>8.3333333333333329E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>31</v>
       </c>
@@ -1081,13 +1247,16 @@
         <v>32</v>
       </c>
       <c r="C31" t="s">
+        <v>82</v>
+      </c>
+      <c r="D31" t="s">
         <v>33</v>
       </c>
-      <c r="D31">
+      <c r="E31">
         <v>1.6000000000000001E-3</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>31</v>
       </c>
@@ -1095,13 +1264,16 @@
         <v>34</v>
       </c>
       <c r="C32" t="s">
+        <v>82</v>
+      </c>
+      <c r="D32" t="s">
         <v>35</v>
       </c>
-      <c r="D32">
+      <c r="E32">
         <v>1.6000000000000001E-3</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>31</v>
       </c>
@@ -1109,13 +1281,16 @@
         <v>36</v>
       </c>
       <c r="C33" t="s">
+        <v>82</v>
+      </c>
+      <c r="D33" t="s">
         <v>37</v>
       </c>
-      <c r="D33">
+      <c r="E33">
         <v>1.6000000000000001E-3</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>31</v>
       </c>
@@ -1123,13 +1298,16 @@
         <v>24</v>
       </c>
       <c r="C34" t="s">
+        <v>82</v>
+      </c>
+      <c r="D34" t="s">
         <v>25</v>
       </c>
-      <c r="D34">
+      <c r="E34">
         <v>1.6000000000000001E-3</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>38</v>
       </c>
@@ -1137,13 +1315,16 @@
         <v>34</v>
       </c>
       <c r="C35" t="s">
+        <v>82</v>
+      </c>
+      <c r="D35" t="s">
         <v>35</v>
       </c>
-      <c r="D35">
+      <c r="E35">
         <v>1.1999999999999999E-3</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>38</v>
       </c>
@@ -1151,13 +1332,16 @@
         <v>36</v>
       </c>
       <c r="C36" t="s">
+        <v>82</v>
+      </c>
+      <c r="D36" t="s">
         <v>37</v>
       </c>
-      <c r="D36">
+      <c r="E36">
         <v>1.1999999999999999E-3</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>38</v>
       </c>
@@ -1165,13 +1349,16 @@
         <v>24</v>
       </c>
       <c r="C37" t="s">
+        <v>82</v>
+      </c>
+      <c r="D37" t="s">
         <v>25</v>
       </c>
-      <c r="D37">
+      <c r="E37">
         <v>1.1999999999999999E-3</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>39</v>
       </c>
@@ -1179,13 +1366,16 @@
         <v>7</v>
       </c>
       <c r="C38" t="s">
+        <v>82</v>
+      </c>
+      <c r="D38" t="s">
         <v>8</v>
       </c>
-      <c r="D38">
+      <c r="E38">
         <v>2E-3</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>39</v>
       </c>
@@ -1193,13 +1383,16 @@
         <v>21</v>
       </c>
       <c r="C39" t="s">
+        <v>82</v>
+      </c>
+      <c r="D39" t="s">
         <v>22</v>
       </c>
-      <c r="D39">
+      <c r="E39">
         <v>2E-3</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>39</v>
       </c>
@@ -1207,13 +1400,16 @@
         <v>40</v>
       </c>
       <c r="C40" t="s">
+        <v>82</v>
+      </c>
+      <c r="D40" t="s">
         <v>41</v>
       </c>
-      <c r="D40">
+      <c r="E40">
         <v>2E-3</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>42</v>
       </c>
@@ -1221,13 +1417,16 @@
         <v>40</v>
       </c>
       <c r="C41" t="s">
+        <v>82</v>
+      </c>
+      <c r="D41" t="s">
         <v>41</v>
       </c>
-      <c r="D41">
+      <c r="E41">
         <v>0.01</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>43</v>
       </c>
@@ -1235,13 +1434,16 @@
         <v>11</v>
       </c>
       <c r="C42" t="s">
+        <v>82</v>
+      </c>
+      <c r="D42" t="s">
         <v>44</v>
       </c>
-      <c r="D42">
+      <c r="E42">
         <v>1.1999999999999999E-3</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>43</v>
       </c>
@@ -1249,13 +1451,16 @@
         <v>45</v>
       </c>
       <c r="C43" t="s">
+        <v>82</v>
+      </c>
+      <c r="D43" t="s">
         <v>46</v>
       </c>
-      <c r="D43">
+      <c r="E43">
         <v>1.1999999999999999E-3</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>47</v>
       </c>
@@ -1263,13 +1468,16 @@
         <v>5</v>
       </c>
       <c r="C44" t="s">
+        <v>82</v>
+      </c>
+      <c r="D44" t="s">
         <v>6</v>
       </c>
-      <c r="D44">
+      <c r="E44">
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>47</v>
       </c>
@@ -1277,13 +1485,16 @@
         <v>7</v>
       </c>
       <c r="C45" t="s">
+        <v>82</v>
+      </c>
+      <c r="D45" t="s">
         <v>8</v>
       </c>
-      <c r="D45">
+      <c r="E45">
         <v>4.3999999999999997E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>48</v>
       </c>
@@ -1291,13 +1502,16 @@
         <v>5</v>
       </c>
       <c r="C46" t="s">
+        <v>82</v>
+      </c>
+      <c r="D46" t="s">
         <v>6</v>
       </c>
-      <c r="D46">
+      <c r="E46">
         <v>0.02</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>48</v>
       </c>
@@ -1305,13 +1519,16 @@
         <v>11</v>
       </c>
       <c r="C47" t="s">
+        <v>82</v>
+      </c>
+      <c r="D47" t="s">
         <v>12</v>
       </c>
-      <c r="D47">
+      <c r="E47">
         <v>0.01</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>48</v>
       </c>
@@ -1319,13 +1536,16 @@
         <v>13</v>
       </c>
       <c r="C48" t="s">
+        <v>82</v>
+      </c>
+      <c r="D48" t="s">
         <v>14</v>
       </c>
-      <c r="D48">
+      <c r="E48">
         <v>0.01</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>48</v>
       </c>
@@ -1333,13 +1553,16 @@
         <v>15</v>
       </c>
       <c r="C49" t="s">
+        <v>82</v>
+      </c>
+      <c r="D49" t="s">
         <v>16</v>
       </c>
-      <c r="D49">
+      <c r="E49">
         <v>0.02</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>48</v>
       </c>
@@ -1347,13 +1570,16 @@
         <v>7</v>
       </c>
       <c r="C50" t="s">
+        <v>82</v>
+      </c>
+      <c r="D50" t="s">
         <v>8</v>
       </c>
-      <c r="D50">
+      <c r="E50">
         <v>8.3333333333333329E-2</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>48</v>
       </c>
@@ -1361,13 +1587,16 @@
         <v>17</v>
       </c>
       <c r="C51" t="s">
+        <v>82</v>
+      </c>
+      <c r="D51" t="s">
         <v>18</v>
       </c>
-      <c r="D51">
+      <c r="E51">
         <v>0.02</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>49</v>
       </c>
@@ -1375,13 +1604,16 @@
         <v>7</v>
       </c>
       <c r="C52" t="s">
+        <v>82</v>
+      </c>
+      <c r="D52" t="s">
         <v>50</v>
       </c>
-      <c r="D52">
+      <c r="E52">
         <v>0.04</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>51</v>
       </c>
@@ -1389,13 +1621,16 @@
         <v>7</v>
       </c>
       <c r="C53" t="s">
+        <v>82</v>
+      </c>
+      <c r="D53" t="s">
         <v>50</v>
       </c>
-      <c r="D53">
+      <c r="E53">
         <v>0.04</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>51</v>
       </c>
@@ -1403,13 +1638,16 @@
         <v>13</v>
       </c>
       <c r="C54" t="s">
+        <v>82</v>
+      </c>
+      <c r="D54" t="s">
         <v>52</v>
       </c>
-      <c r="D54">
+      <c r="E54">
         <v>2.1999999999999999E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>51</v>
       </c>
@@ -1417,13 +1655,16 @@
         <v>15</v>
       </c>
       <c r="C55" t="s">
+        <v>82</v>
+      </c>
+      <c r="D55" t="s">
         <v>53</v>
       </c>
-      <c r="D55">
+      <c r="E55">
         <v>2.1999999999999999E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>51</v>
       </c>
@@ -1431,13 +1672,16 @@
         <v>17</v>
       </c>
       <c r="C56" t="s">
+        <v>82</v>
+      </c>
+      <c r="D56" t="s">
         <v>18</v>
       </c>
-      <c r="D56">
+      <c r="E56">
         <v>3.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>51</v>
       </c>
@@ -1445,13 +1689,16 @@
         <v>21</v>
       </c>
       <c r="C57" t="s">
+        <v>82</v>
+      </c>
+      <c r="D57" t="s">
         <v>22</v>
       </c>
-      <c r="D57">
+      <c r="E57">
         <v>1.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>54</v>
       </c>
@@ -1459,13 +1706,16 @@
         <v>5</v>
       </c>
       <c r="C58" t="s">
+        <v>82</v>
+      </c>
+      <c r="D58" t="s">
         <v>6</v>
       </c>
-      <c r="D58">
+      <c r="E58">
         <v>0.02</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>54</v>
       </c>
@@ -1473,13 +1723,16 @@
         <v>11</v>
       </c>
       <c r="C59" t="s">
+        <v>82</v>
+      </c>
+      <c r="D59" t="s">
         <v>12</v>
       </c>
-      <c r="D59">
+      <c r="E59">
         <v>0.01</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>54</v>
       </c>
@@ -1487,13 +1740,16 @@
         <v>13</v>
       </c>
       <c r="C60" t="s">
+        <v>82</v>
+      </c>
+      <c r="D60" t="s">
         <v>14</v>
       </c>
-      <c r="D60">
+      <c r="E60">
         <v>0.01</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>54</v>
       </c>
@@ -1501,13 +1757,16 @@
         <v>15</v>
       </c>
       <c r="C61" t="s">
+        <v>82</v>
+      </c>
+      <c r="D61" t="s">
         <v>16</v>
       </c>
-      <c r="D61">
+      <c r="E61">
         <v>0.02</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>54</v>
       </c>
@@ -1515,13 +1774,16 @@
         <v>7</v>
       </c>
       <c r="C62" t="s">
+        <v>82</v>
+      </c>
+      <c r="D62" t="s">
         <v>8</v>
       </c>
-      <c r="D62">
+      <c r="E62">
         <v>8.3333333333333329E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>54</v>
       </c>
@@ -1529,13 +1791,16 @@
         <v>17</v>
       </c>
       <c r="C63" t="s">
+        <v>82</v>
+      </c>
+      <c r="D63" t="s">
         <v>18</v>
       </c>
-      <c r="D63">
+      <c r="E63">
         <v>0.02</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>55</v>
       </c>
@@ -1543,13 +1808,16 @@
         <v>5</v>
       </c>
       <c r="C64" t="s">
+        <v>82</v>
+      </c>
+      <c r="D64" t="s">
         <v>6</v>
       </c>
-      <c r="D64">
+      <c r="E64">
         <v>0.02</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>55</v>
       </c>
@@ -1557,13 +1825,16 @@
         <v>11</v>
       </c>
       <c r="C65" t="s">
+        <v>82</v>
+      </c>
+      <c r="D65" t="s">
         <v>12</v>
       </c>
-      <c r="D65">
+      <c r="E65">
         <v>0.01</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>55</v>
       </c>
@@ -1571,13 +1842,16 @@
         <v>13</v>
       </c>
       <c r="C66" t="s">
+        <v>82</v>
+      </c>
+      <c r="D66" t="s">
         <v>14</v>
       </c>
-      <c r="D66">
+      <c r="E66">
         <v>0.01</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>55</v>
       </c>
@@ -1585,13 +1859,16 @@
         <v>15</v>
       </c>
       <c r="C67" t="s">
+        <v>82</v>
+      </c>
+      <c r="D67" t="s">
         <v>16</v>
       </c>
-      <c r="D67">
+      <c r="E67">
         <v>0.02</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>55</v>
       </c>
@@ -1599,13 +1876,16 @@
         <v>7</v>
       </c>
       <c r="C68" t="s">
+        <v>82</v>
+      </c>
+      <c r="D68" t="s">
         <v>8</v>
       </c>
-      <c r="D68">
+      <c r="E68">
         <v>8.3333333333333329E-2</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>55</v>
       </c>
@@ -1613,13 +1893,16 @@
         <v>17</v>
       </c>
       <c r="C69" t="s">
+        <v>82</v>
+      </c>
+      <c r="D69" t="s">
         <v>18</v>
       </c>
-      <c r="D69">
+      <c r="E69">
         <v>0.02</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>56</v>
       </c>
@@ -1627,13 +1910,16 @@
         <v>57</v>
       </c>
       <c r="C70" t="s">
+        <v>82</v>
+      </c>
+      <c r="D70" t="s">
         <v>58</v>
       </c>
-      <c r="D70">
+      <c r="E70">
         <v>0.25</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>56</v>
       </c>
@@ -1641,13 +1927,16 @@
         <v>59</v>
       </c>
       <c r="C71" t="s">
+        <v>82</v>
+      </c>
+      <c r="D71" t="s">
         <v>60</v>
       </c>
-      <c r="D71">
+      <c r="E71">
         <v>1.666666666666667E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>56</v>
       </c>
@@ -1655,13 +1944,16 @@
         <v>24</v>
       </c>
       <c r="C72" t="s">
+        <v>82</v>
+      </c>
+      <c r="D72" t="s">
         <v>25</v>
       </c>
-      <c r="D72">
+      <c r="E72">
         <v>0.4</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>61</v>
       </c>
@@ -1669,13 +1961,16 @@
         <v>57</v>
       </c>
       <c r="C73" t="s">
+        <v>82</v>
+      </c>
+      <c r="D73" t="s">
         <v>58</v>
       </c>
-      <c r="D73">
+      <c r="E73">
         <v>0.25</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>61</v>
       </c>
@@ -1683,13 +1978,16 @@
         <v>59</v>
       </c>
       <c r="C74" t="s">
+        <v>82</v>
+      </c>
+      <c r="D74" t="s">
         <v>60</v>
       </c>
-      <c r="D74">
+      <c r="E74">
         <v>1.666666666666667E-2</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>61</v>
       </c>
@@ -1697,13 +1995,16 @@
         <v>24</v>
       </c>
       <c r="C75" t="s">
+        <v>82</v>
+      </c>
+      <c r="D75" t="s">
         <v>25</v>
       </c>
-      <c r="D75">
+      <c r="E75">
         <v>0.4</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>62</v>
       </c>
@@ -1711,13 +2012,16 @@
         <v>45</v>
       </c>
       <c r="C76" t="s">
+        <v>82</v>
+      </c>
+      <c r="D76" t="s">
         <v>63</v>
       </c>
-      <c r="D76">
+      <c r="E76">
         <v>1.8749999999999999E-3</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>64</v>
       </c>
@@ -1725,13 +2029,16 @@
         <v>45</v>
       </c>
       <c r="C77" t="s">
+        <v>82</v>
+      </c>
+      <c r="D77" t="s">
         <v>63</v>
       </c>
-      <c r="D77">
+      <c r="E77">
         <v>1.8749999999999999E-3</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>65</v>
       </c>
@@ -1739,13 +2046,16 @@
         <v>13</v>
       </c>
       <c r="C78" t="s">
+        <v>82</v>
+      </c>
+      <c r="D78" t="s">
         <v>14</v>
       </c>
-      <c r="D78">
+      <c r="E78">
         <v>0.02</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>65</v>
       </c>
@@ -1753,13 +2063,16 @@
         <v>15</v>
       </c>
       <c r="C79" t="s">
+        <v>82</v>
+      </c>
+      <c r="D79" t="s">
         <v>16</v>
       </c>
-      <c r="D79">
+      <c r="E79">
         <v>0.04</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>65</v>
       </c>
@@ -1767,13 +2080,16 @@
         <v>21</v>
       </c>
       <c r="C80" t="s">
+        <v>82</v>
+      </c>
+      <c r="D80" t="s">
         <v>22</v>
       </c>
-      <c r="D80">
+      <c r="E80">
         <v>0.04</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>65</v>
       </c>
@@ -1781,13 +2097,16 @@
         <v>7</v>
       </c>
       <c r="C81" t="s">
+        <v>82</v>
+      </c>
+      <c r="D81" t="s">
         <v>8</v>
       </c>
-      <c r="D81">
+      <c r="E81">
         <v>8.3333333333333329E-2</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>65</v>
       </c>
@@ -1795,13 +2114,16 @@
         <v>17</v>
       </c>
       <c r="C82" t="s">
+        <v>82</v>
+      </c>
+      <c r="D82" t="s">
         <v>18</v>
       </c>
-      <c r="D82">
+      <c r="E82">
         <v>3.3000000000000002E-2</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>66</v>
       </c>
@@ -1809,13 +2131,16 @@
         <v>24</v>
       </c>
       <c r="C83" t="s">
+        <v>82</v>
+      </c>
+      <c r="D83" t="s">
         <v>25</v>
       </c>
-      <c r="D83">
+      <c r="E83">
         <v>6.2827225130890049E-2</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>66</v>
       </c>
@@ -1823,13 +2148,16 @@
         <v>26</v>
       </c>
       <c r="C84" t="s">
+        <v>82</v>
+      </c>
+      <c r="D84" t="s">
         <v>27</v>
       </c>
-      <c r="D84">
+      <c r="E84">
         <v>6.2827225130890049E-2</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>66</v>
       </c>
@@ -1837,13 +2165,16 @@
         <v>28</v>
       </c>
       <c r="C85" t="s">
+        <v>82</v>
+      </c>
+      <c r="D85" t="s">
         <v>29</v>
       </c>
-      <c r="D85">
+      <c r="E85">
         <v>0.1256544502617801</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>66</v>
       </c>
@@ -1851,13 +2182,16 @@
         <v>7</v>
       </c>
       <c r="C86" t="s">
+        <v>82</v>
+      </c>
+      <c r="D86" t="s">
         <v>8</v>
       </c>
-      <c r="D86">
+      <c r="E86">
         <v>8.3333333333333329E-2</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>67</v>
       </c>
@@ -1865,13 +2199,16 @@
         <v>24</v>
       </c>
       <c r="C87" t="s">
+        <v>82</v>
+      </c>
+      <c r="D87" t="s">
         <v>25</v>
       </c>
-      <c r="D87">
+      <c r="E87">
         <v>6.2827225130890049E-2</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>67</v>
       </c>
@@ -1879,13 +2216,16 @@
         <v>26</v>
       </c>
       <c r="C88" t="s">
+        <v>82</v>
+      </c>
+      <c r="D88" t="s">
         <v>27</v>
       </c>
-      <c r="D88">
+      <c r="E88">
         <v>6.2827225130890049E-2</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>67</v>
       </c>
@@ -1893,13 +2233,16 @@
         <v>28</v>
       </c>
       <c r="C89" t="s">
+        <v>82</v>
+      </c>
+      <c r="D89" t="s">
         <v>29</v>
       </c>
-      <c r="D89">
+      <c r="E89">
         <v>0.1256544502617801</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>67</v>
       </c>
@@ -1907,13 +2250,16 @@
         <v>7</v>
       </c>
       <c r="C90" t="s">
+        <v>82</v>
+      </c>
+      <c r="D90" t="s">
         <v>8</v>
       </c>
-      <c r="D90">
+      <c r="E90">
         <v>8.3333333333333329E-2</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>68</v>
       </c>
@@ -1921,13 +2267,16 @@
         <v>32</v>
       </c>
       <c r="C91" t="s">
+        <v>82</v>
+      </c>
+      <c r="D91" t="s">
         <v>33</v>
       </c>
-      <c r="D91">
+      <c r="E91">
         <v>1.6000000000000001E-3</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>68</v>
       </c>
@@ -1935,13 +2284,16 @@
         <v>34</v>
       </c>
       <c r="C92" t="s">
+        <v>82</v>
+      </c>
+      <c r="D92" t="s">
         <v>35</v>
       </c>
-      <c r="D92">
+      <c r="E92">
         <v>1.6000000000000001E-3</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>68</v>
       </c>
@@ -1949,13 +2301,16 @@
         <v>36</v>
       </c>
       <c r="C93" t="s">
+        <v>82</v>
+      </c>
+      <c r="D93" t="s">
         <v>37</v>
       </c>
-      <c r="D93">
+      <c r="E93">
         <v>1.6000000000000001E-3</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>68</v>
       </c>
@@ -1963,13 +2318,16 @@
         <v>24</v>
       </c>
       <c r="C94" t="s">
+        <v>82</v>
+      </c>
+      <c r="D94" t="s">
         <v>25</v>
       </c>
-      <c r="D94">
+      <c r="E94">
         <v>1.6000000000000001E-3</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>69</v>
       </c>
@@ -1977,13 +2335,16 @@
         <v>34</v>
       </c>
       <c r="C95" t="s">
+        <v>82</v>
+      </c>
+      <c r="D95" t="s">
         <v>35</v>
       </c>
-      <c r="D95">
+      <c r="E95">
         <v>1.1999999999999999E-3</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>69</v>
       </c>
@@ -1991,13 +2352,16 @@
         <v>36</v>
       </c>
       <c r="C96" t="s">
+        <v>82</v>
+      </c>
+      <c r="D96" t="s">
         <v>37</v>
       </c>
-      <c r="D96">
+      <c r="E96">
         <v>1.1999999999999999E-3</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>69</v>
       </c>
@@ -2005,13 +2369,16 @@
         <v>24</v>
       </c>
       <c r="C97" t="s">
+        <v>82</v>
+      </c>
+      <c r="D97" t="s">
         <v>25</v>
       </c>
-      <c r="D97">
+      <c r="E97">
         <v>1.1999999999999999E-3</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>70</v>
       </c>
@@ -2019,13 +2386,16 @@
         <v>34</v>
       </c>
       <c r="C98" t="s">
+        <v>82</v>
+      </c>
+      <c r="D98" t="s">
         <v>35</v>
       </c>
-      <c r="D98">
+      <c r="E98">
         <v>1.1999999999999999E-3</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>70</v>
       </c>
@@ -2033,13 +2403,16 @@
         <v>36</v>
       </c>
       <c r="C99" t="s">
+        <v>82</v>
+      </c>
+      <c r="D99" t="s">
         <v>37</v>
       </c>
-      <c r="D99">
+      <c r="E99">
         <v>1.1999999999999999E-3</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>70</v>
       </c>
@@ -2047,13 +2420,16 @@
         <v>24</v>
       </c>
       <c r="C100" t="s">
+        <v>82</v>
+      </c>
+      <c r="D100" t="s">
         <v>25</v>
       </c>
-      <c r="D100">
+      <c r="E100">
         <v>1.1999999999999999E-3</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>71</v>
       </c>
@@ -2061,13 +2437,16 @@
         <v>21</v>
       </c>
       <c r="C101" t="s">
+        <v>82</v>
+      </c>
+      <c r="D101" t="s">
         <v>72</v>
       </c>
-      <c r="D101">
+      <c r="E101">
         <v>2E-3</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>71</v>
       </c>
@@ -2075,13 +2454,16 @@
         <v>21</v>
       </c>
       <c r="C102" t="s">
+        <v>82</v>
+      </c>
+      <c r="D102" t="s">
         <v>22</v>
       </c>
-      <c r="D102">
+      <c r="E102">
         <v>2E-3</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>71</v>
       </c>
@@ -2089,13 +2471,16 @@
         <v>7</v>
       </c>
       <c r="C103" t="s">
+        <v>82</v>
+      </c>
+      <c r="D103" t="s">
         <v>8</v>
       </c>
-      <c r="D103">
+      <c r="E103">
         <v>2E-3</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>73</v>
       </c>
@@ -2103,13 +2488,16 @@
         <v>57</v>
       </c>
       <c r="C104" t="s">
+        <v>82</v>
+      </c>
+      <c r="D104" t="s">
         <v>58</v>
       </c>
-      <c r="D104">
+      <c r="E104">
         <v>0.25</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>73</v>
       </c>
@@ -2117,13 +2505,16 @@
         <v>59</v>
       </c>
       <c r="C105" t="s">
+        <v>82</v>
+      </c>
+      <c r="D105" t="s">
         <v>60</v>
       </c>
-      <c r="D105">
+      <c r="E105">
         <v>1.666666666666667E-2</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>73</v>
       </c>
@@ -2131,13 +2522,16 @@
         <v>24</v>
       </c>
       <c r="C106" t="s">
+        <v>82</v>
+      </c>
+      <c r="D106" t="s">
         <v>25</v>
       </c>
-      <c r="D106">
+      <c r="E106">
         <v>0.4</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>74</v>
       </c>
@@ -2145,13 +2539,16 @@
         <v>57</v>
       </c>
       <c r="C107" t="s">
+        <v>82</v>
+      </c>
+      <c r="D107" t="s">
         <v>58</v>
       </c>
-      <c r="D107">
+      <c r="E107">
         <v>0.25</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>74</v>
       </c>
@@ -2159,13 +2556,16 @@
         <v>59</v>
       </c>
       <c r="C108" t="s">
+        <v>82</v>
+      </c>
+      <c r="D108" t="s">
         <v>60</v>
       </c>
-      <c r="D108">
+      <c r="E108">
         <v>1.666666666666667E-2</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>74</v>
       </c>
@@ -2173,13 +2573,16 @@
         <v>24</v>
       </c>
       <c r="C109" t="s">
+        <v>82</v>
+      </c>
+      <c r="D109" t="s">
         <v>25</v>
       </c>
-      <c r="D109">
+      <c r="E109">
         <v>0.4</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>75</v>
       </c>
@@ -2187,13 +2590,16 @@
         <v>57</v>
       </c>
       <c r="C110" t="s">
+        <v>82</v>
+      </c>
+      <c r="D110" t="s">
         <v>58</v>
       </c>
-      <c r="D110">
+      <c r="E110">
         <v>0.25</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>75</v>
       </c>
@@ -2201,13 +2607,16 @@
         <v>59</v>
       </c>
       <c r="C111" t="s">
+        <v>82</v>
+      </c>
+      <c r="D111" t="s">
         <v>60</v>
       </c>
-      <c r="D111">
+      <c r="E111">
         <v>1.666666666666667E-2</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>75</v>
       </c>
@@ -2215,13 +2624,16 @@
         <v>24</v>
       </c>
       <c r="C112" t="s">
+        <v>82</v>
+      </c>
+      <c r="D112" t="s">
         <v>25</v>
       </c>
-      <c r="D112">
+      <c r="E112">
         <v>0.4</v>
       </c>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>76</v>
       </c>
@@ -2229,13 +2641,16 @@
         <v>57</v>
       </c>
       <c r="C113" t="s">
+        <v>82</v>
+      </c>
+      <c r="D113" t="s">
         <v>58</v>
       </c>
-      <c r="D113">
+      <c r="E113">
         <v>0.25</v>
       </c>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>76</v>
       </c>
@@ -2243,13 +2658,16 @@
         <v>59</v>
       </c>
       <c r="C114" t="s">
+        <v>82</v>
+      </c>
+      <c r="D114" t="s">
         <v>60</v>
       </c>
-      <c r="D114">
+      <c r="E114">
         <v>1.666666666666667E-2</v>
       </c>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>76</v>
       </c>
@@ -2257,13 +2675,16 @@
         <v>24</v>
       </c>
       <c r="C115" t="s">
+        <v>82</v>
+      </c>
+      <c r="D115" t="s">
         <v>25</v>
       </c>
-      <c r="D115">
+      <c r="E115">
         <v>0.4</v>
       </c>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>77</v>
       </c>
@@ -2271,13 +2692,16 @@
         <v>78</v>
       </c>
       <c r="C116" t="s">
+        <v>82</v>
+      </c>
+      <c r="D116" t="s">
         <v>79</v>
       </c>
-      <c r="D116">
+      <c r="E116">
         <v>0.15</v>
       </c>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>80</v>
       </c>
@@ -2285,13 +2709,16 @@
         <v>57</v>
       </c>
       <c r="C117" t="s">
+        <v>82</v>
+      </c>
+      <c r="D117" t="s">
         <v>58</v>
       </c>
-      <c r="D117">
+      <c r="E117">
         <v>0.25</v>
       </c>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>80</v>
       </c>
@@ -2299,13 +2726,16 @@
         <v>59</v>
       </c>
       <c r="C118" t="s">
+        <v>82</v>
+      </c>
+      <c r="D118" t="s">
         <v>60</v>
       </c>
-      <c r="D118">
+      <c r="E118">
         <v>1.666666666666667E-2</v>
       </c>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>80</v>
       </c>
@@ -2313,10 +2743,1764 @@
         <v>24</v>
       </c>
       <c r="C119" t="s">
+        <v>82</v>
+      </c>
+      <c r="D119" t="s">
         <v>25</v>
       </c>
-      <c r="D119">
+      <c r="E119">
         <v>0.4</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>4</v>
+      </c>
+      <c r="B120" t="s">
+        <v>83</v>
+      </c>
+      <c r="C120" t="s">
+        <v>84</v>
+      </c>
+      <c r="D120" t="s">
+        <v>103</v>
+      </c>
+      <c r="E120">
+        <v>3.3333333333333333E-2</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>4</v>
+      </c>
+      <c r="B121" t="s">
+        <v>87</v>
+      </c>
+      <c r="C121" t="s">
+        <v>84</v>
+      </c>
+      <c r="D121" t="s">
+        <v>104</v>
+      </c>
+      <c r="E121">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>9</v>
+      </c>
+      <c r="B122" t="s">
+        <v>83</v>
+      </c>
+      <c r="C122" t="s">
+        <v>84</v>
+      </c>
+      <c r="D122" t="s">
+        <v>103</v>
+      </c>
+      <c r="E122">
+        <v>3.3333333333333333E-2</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>9</v>
+      </c>
+      <c r="B123" t="s">
+        <v>87</v>
+      </c>
+      <c r="C123" t="s">
+        <v>84</v>
+      </c>
+      <c r="D123" t="s">
+        <v>104</v>
+      </c>
+      <c r="E123">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>10</v>
+      </c>
+      <c r="B124" t="s">
+        <v>83</v>
+      </c>
+      <c r="C124" t="s">
+        <v>84</v>
+      </c>
+      <c r="D124" t="s">
+        <v>103</v>
+      </c>
+      <c r="E124">
+        <v>2.6666666666666668E-2</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>10</v>
+      </c>
+      <c r="B125" t="s">
+        <v>87</v>
+      </c>
+      <c r="C125" t="s">
+        <v>84</v>
+      </c>
+      <c r="D125" t="s">
+        <v>104</v>
+      </c>
+      <c r="E125">
+        <v>0.10666666666666667</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>19</v>
+      </c>
+      <c r="B126" t="s">
+        <v>83</v>
+      </c>
+      <c r="C126" t="s">
+        <v>84</v>
+      </c>
+      <c r="D126" t="s">
+        <v>103</v>
+      </c>
+      <c r="E126">
+        <v>2.6666666666666668E-2</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>19</v>
+      </c>
+      <c r="B127" t="s">
+        <v>87</v>
+      </c>
+      <c r="C127" t="s">
+        <v>84</v>
+      </c>
+      <c r="D127" t="s">
+        <v>104</v>
+      </c>
+      <c r="E127">
+        <v>0.10666666666666667</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>20</v>
+      </c>
+      <c r="B128" t="s">
+        <v>83</v>
+      </c>
+      <c r="C128" t="s">
+        <v>84</v>
+      </c>
+      <c r="D128" t="s">
+        <v>103</v>
+      </c>
+      <c r="E128">
+        <v>5.3333333333333337E-2</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>20</v>
+      </c>
+      <c r="B129" t="s">
+        <v>87</v>
+      </c>
+      <c r="C129" t="s">
+        <v>84</v>
+      </c>
+      <c r="D129" t="s">
+        <v>104</v>
+      </c>
+      <c r="E129">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>23</v>
+      </c>
+      <c r="B130" t="s">
+        <v>83</v>
+      </c>
+      <c r="C130" t="s">
+        <v>84</v>
+      </c>
+      <c r="D130" t="s">
+        <v>103</v>
+      </c>
+      <c r="E130">
+        <v>0.41884816753926701</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>23</v>
+      </c>
+      <c r="B131" t="s">
+        <v>87</v>
+      </c>
+      <c r="C131" t="s">
+        <v>84</v>
+      </c>
+      <c r="D131" t="s">
+        <v>104</v>
+      </c>
+      <c r="E131">
+        <v>1.256544502617801</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>30</v>
+      </c>
+      <c r="B132" t="s">
+        <v>83</v>
+      </c>
+      <c r="C132" t="s">
+        <v>84</v>
+      </c>
+      <c r="D132" t="s">
+        <v>103</v>
+      </c>
+      <c r="E132">
+        <v>0.41884816753926701</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>30</v>
+      </c>
+      <c r="B133" t="s">
+        <v>87</v>
+      </c>
+      <c r="C133" t="s">
+        <v>84</v>
+      </c>
+      <c r="D133" t="s">
+        <v>104</v>
+      </c>
+      <c r="E133">
+        <v>1.256544502617801</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>31</v>
+      </c>
+      <c r="B134" t="s">
+        <v>83</v>
+      </c>
+      <c r="C134" t="s">
+        <v>84</v>
+      </c>
+      <c r="D134" t="s">
+        <v>103</v>
+      </c>
+      <c r="E134">
+        <v>4.7999999999999996E-3</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
+        <v>31</v>
+      </c>
+      <c r="B135" t="s">
+        <v>87</v>
+      </c>
+      <c r="C135" t="s">
+        <v>84</v>
+      </c>
+      <c r="D135" t="s">
+        <v>104</v>
+      </c>
+      <c r="E135">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
+        <v>38</v>
+      </c>
+      <c r="B136" t="s">
+        <v>83</v>
+      </c>
+      <c r="C136" t="s">
+        <v>84</v>
+      </c>
+      <c r="D136" t="s">
+        <v>103</v>
+      </c>
+      <c r="E136">
+        <v>4.7999999999999996E-3</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
+        <v>38</v>
+      </c>
+      <c r="B137" t="s">
+        <v>87</v>
+      </c>
+      <c r="C137" t="s">
+        <v>84</v>
+      </c>
+      <c r="D137" t="s">
+        <v>104</v>
+      </c>
+      <c r="E137">
+        <v>3.2000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
+        <v>39</v>
+      </c>
+      <c r="B138" t="s">
+        <v>83</v>
+      </c>
+      <c r="C138" t="s">
+        <v>84</v>
+      </c>
+      <c r="D138" t="s">
+        <v>103</v>
+      </c>
+      <c r="E138">
+        <v>2.6666666666666666E-3</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
+        <v>39</v>
+      </c>
+      <c r="B139" t="s">
+        <v>87</v>
+      </c>
+      <c r="C139" t="s">
+        <v>84</v>
+      </c>
+      <c r="D139" t="s">
+        <v>104</v>
+      </c>
+      <c r="E139">
+        <v>1.6E-2</v>
+      </c>
+    </row>
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
+        <v>42</v>
+      </c>
+      <c r="B140" t="s">
+        <v>83</v>
+      </c>
+      <c r="C140" t="s">
+        <v>84</v>
+      </c>
+      <c r="D140" t="s">
+        <v>103</v>
+      </c>
+      <c r="E140">
+        <v>1.3333333333333334E-2</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A141" t="s">
+        <v>42</v>
+      </c>
+      <c r="B141" t="s">
+        <v>87</v>
+      </c>
+      <c r="C141" t="s">
+        <v>84</v>
+      </c>
+      <c r="D141" t="s">
+        <v>104</v>
+      </c>
+      <c r="E141">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
+        <v>85</v>
+      </c>
+      <c r="B142" t="s">
+        <v>83</v>
+      </c>
+      <c r="C142" t="s">
+        <v>84</v>
+      </c>
+      <c r="D142" t="s">
+        <v>103</v>
+      </c>
+      <c r="E142">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
+        <v>85</v>
+      </c>
+      <c r="B143" t="s">
+        <v>87</v>
+      </c>
+      <c r="C143" t="s">
+        <v>84</v>
+      </c>
+      <c r="D143" t="s">
+        <v>104</v>
+      </c>
+      <c r="E143">
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
+        <v>86</v>
+      </c>
+      <c r="B144" t="s">
+        <v>83</v>
+      </c>
+      <c r="C144" t="s">
+        <v>84</v>
+      </c>
+      <c r="D144" t="s">
+        <v>103</v>
+      </c>
+      <c r="E144">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
+        <v>86</v>
+      </c>
+      <c r="B145" t="s">
+        <v>87</v>
+      </c>
+      <c r="C145" t="s">
+        <v>84</v>
+      </c>
+      <c r="D145" t="s">
+        <v>104</v>
+      </c>
+      <c r="E145">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
+        <v>43</v>
+      </c>
+      <c r="B146" t="s">
+        <v>87</v>
+      </c>
+      <c r="C146" t="s">
+        <v>84</v>
+      </c>
+      <c r="D146" t="s">
+        <v>104</v>
+      </c>
+      <c r="E146">
+        <v>6.4000000000000003E-3</v>
+      </c>
+    </row>
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A147" t="s">
+        <v>47</v>
+      </c>
+      <c r="B147" t="s">
+        <v>83</v>
+      </c>
+      <c r="C147" t="s">
+        <v>84</v>
+      </c>
+      <c r="D147" t="s">
+        <v>103</v>
+      </c>
+      <c r="E147">
+        <v>3.3333333333333333E-2</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A148" t="s">
+        <v>47</v>
+      </c>
+      <c r="B148" t="s">
+        <v>87</v>
+      </c>
+      <c r="C148" t="s">
+        <v>84</v>
+      </c>
+      <c r="D148" t="s">
+        <v>104</v>
+      </c>
+      <c r="E148">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A149" t="s">
+        <v>48</v>
+      </c>
+      <c r="B149" t="s">
+        <v>83</v>
+      </c>
+      <c r="C149" t="s">
+        <v>84</v>
+      </c>
+      <c r="D149" t="s">
+        <v>103</v>
+      </c>
+      <c r="E149">
+        <v>2.6666666666666668E-2</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A150" t="s">
+        <v>48</v>
+      </c>
+      <c r="B150" t="s">
+        <v>87</v>
+      </c>
+      <c r="C150" t="s">
+        <v>84</v>
+      </c>
+      <c r="D150" t="s">
+        <v>104</v>
+      </c>
+      <c r="E150">
+        <v>0.10666666666666667</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A151" t="s">
+        <v>49</v>
+      </c>
+      <c r="B151" t="s">
+        <v>87</v>
+      </c>
+      <c r="C151" t="s">
+        <v>84</v>
+      </c>
+      <c r="D151" t="s">
+        <v>104</v>
+      </c>
+      <c r="E151">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A152" t="s">
+        <v>49</v>
+      </c>
+      <c r="B152" t="s">
+        <v>87</v>
+      </c>
+      <c r="C152" t="s">
+        <v>84</v>
+      </c>
+      <c r="D152" t="s">
+        <v>104</v>
+      </c>
+      <c r="E152">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
+        <v>51</v>
+      </c>
+      <c r="B153" t="s">
+        <v>87</v>
+      </c>
+      <c r="C153" t="s">
+        <v>84</v>
+      </c>
+      <c r="D153" t="s">
+        <v>104</v>
+      </c>
+      <c r="E153">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>51</v>
+      </c>
+      <c r="B154" t="s">
+        <v>87</v>
+      </c>
+      <c r="C154" t="s">
+        <v>84</v>
+      </c>
+      <c r="D154" t="s">
+        <v>104</v>
+      </c>
+      <c r="E154">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
+        <v>54</v>
+      </c>
+      <c r="B155" t="s">
+        <v>83</v>
+      </c>
+      <c r="C155" t="s">
+        <v>84</v>
+      </c>
+      <c r="D155" t="s">
+        <v>103</v>
+      </c>
+      <c r="E155">
+        <v>2.6666666666666668E-2</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A156" t="s">
+        <v>54</v>
+      </c>
+      <c r="B156" t="s">
+        <v>87</v>
+      </c>
+      <c r="C156" t="s">
+        <v>84</v>
+      </c>
+      <c r="D156" t="s">
+        <v>104</v>
+      </c>
+      <c r="E156">
+        <v>0.10666666666666667</v>
+      </c>
+    </row>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A157" t="s">
+        <v>55</v>
+      </c>
+      <c r="B157" t="s">
+        <v>83</v>
+      </c>
+      <c r="C157" t="s">
+        <v>84</v>
+      </c>
+      <c r="D157" t="s">
+        <v>103</v>
+      </c>
+      <c r="E157">
+        <v>2.6666666666666668E-2</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A158" t="s">
+        <v>55</v>
+      </c>
+      <c r="B158" t="s">
+        <v>87</v>
+      </c>
+      <c r="C158" t="s">
+        <v>84</v>
+      </c>
+      <c r="D158" t="s">
+        <v>104</v>
+      </c>
+      <c r="E158">
+        <v>0.10666666666666667</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
+        <v>88</v>
+      </c>
+      <c r="B159" t="s">
+        <v>83</v>
+      </c>
+      <c r="C159" t="s">
+        <v>84</v>
+      </c>
+      <c r="D159" t="s">
+        <v>103</v>
+      </c>
+      <c r="E159">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A160" t="s">
+        <v>88</v>
+      </c>
+      <c r="B160" t="s">
+        <v>87</v>
+      </c>
+      <c r="C160" t="s">
+        <v>84</v>
+      </c>
+      <c r="D160" t="s">
+        <v>104</v>
+      </c>
+      <c r="E160">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A161" t="s">
+        <v>89</v>
+      </c>
+      <c r="B161" t="s">
+        <v>83</v>
+      </c>
+      <c r="C161" t="s">
+        <v>84</v>
+      </c>
+      <c r="D161" t="s">
+        <v>103</v>
+      </c>
+      <c r="E161">
+        <v>0.24</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A162" t="s">
+        <v>89</v>
+      </c>
+      <c r="B162" t="s">
+        <v>87</v>
+      </c>
+      <c r="C162" t="s">
+        <v>84</v>
+      </c>
+      <c r="D162" t="s">
+        <v>104</v>
+      </c>
+      <c r="E162">
+        <v>0.24</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A163" t="s">
+        <v>90</v>
+      </c>
+      <c r="B163" t="s">
+        <v>83</v>
+      </c>
+      <c r="C163" t="s">
+        <v>84</v>
+      </c>
+      <c r="D163" t="s">
+        <v>103</v>
+      </c>
+      <c r="E163">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A164" t="s">
+        <v>90</v>
+      </c>
+      <c r="B164" t="s">
+        <v>87</v>
+      </c>
+      <c r="C164" t="s">
+        <v>84</v>
+      </c>
+      <c r="D164" t="s">
+        <v>104</v>
+      </c>
+      <c r="E164">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A165" t="s">
+        <v>91</v>
+      </c>
+      <c r="B165" t="s">
+        <v>83</v>
+      </c>
+      <c r="C165" t="s">
+        <v>84</v>
+      </c>
+      <c r="D165" t="s">
+        <v>103</v>
+      </c>
+      <c r="E165">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A166" t="s">
+        <v>91</v>
+      </c>
+      <c r="B166" t="s">
+        <v>87</v>
+      </c>
+      <c r="C166" t="s">
+        <v>84</v>
+      </c>
+      <c r="D166" t="s">
+        <v>104</v>
+      </c>
+      <c r="E166">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A167" t="s">
+        <v>92</v>
+      </c>
+      <c r="B167" t="s">
+        <v>83</v>
+      </c>
+      <c r="C167" t="s">
+        <v>84</v>
+      </c>
+      <c r="D167" t="s">
+        <v>103</v>
+      </c>
+      <c r="E167">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A168" t="s">
+        <v>92</v>
+      </c>
+      <c r="B168" t="s">
+        <v>87</v>
+      </c>
+      <c r="C168" t="s">
+        <v>84</v>
+      </c>
+      <c r="D168" t="s">
+        <v>104</v>
+      </c>
+      <c r="E168">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A169" t="s">
+        <v>56</v>
+      </c>
+      <c r="B169" t="s">
+        <v>83</v>
+      </c>
+      <c r="C169" t="s">
+        <v>84</v>
+      </c>
+      <c r="D169" t="s">
+        <v>103</v>
+      </c>
+      <c r="E169">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A170" t="s">
+        <v>56</v>
+      </c>
+      <c r="B170" t="s">
+        <v>87</v>
+      </c>
+      <c r="C170" t="s">
+        <v>84</v>
+      </c>
+      <c r="D170" t="s">
+        <v>104</v>
+      </c>
+      <c r="E170">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A171" t="s">
+        <v>61</v>
+      </c>
+      <c r="B171" t="s">
+        <v>83</v>
+      </c>
+      <c r="C171" t="s">
+        <v>84</v>
+      </c>
+      <c r="D171" t="s">
+        <v>103</v>
+      </c>
+      <c r="E171">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A172" t="s">
+        <v>61</v>
+      </c>
+      <c r="B172" t="s">
+        <v>87</v>
+      </c>
+      <c r="C172" t="s">
+        <v>84</v>
+      </c>
+      <c r="D172" t="s">
+        <v>104</v>
+      </c>
+      <c r="E172">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A173" t="s">
+        <v>93</v>
+      </c>
+      <c r="B173" t="s">
+        <v>83</v>
+      </c>
+      <c r="C173" t="s">
+        <v>84</v>
+      </c>
+      <c r="D173" t="s">
+        <v>103</v>
+      </c>
+      <c r="E173">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A174" t="s">
+        <v>93</v>
+      </c>
+      <c r="B174" t="s">
+        <v>87</v>
+      </c>
+      <c r="C174" t="s">
+        <v>84</v>
+      </c>
+      <c r="D174" t="s">
+        <v>104</v>
+      </c>
+      <c r="E174">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A175" t="s">
+        <v>62</v>
+      </c>
+      <c r="B175" t="s">
+        <v>87</v>
+      </c>
+      <c r="C175" t="s">
+        <v>84</v>
+      </c>
+      <c r="D175" t="s">
+        <v>104</v>
+      </c>
+      <c r="E175">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A176" t="s">
+        <v>62</v>
+      </c>
+      <c r="B176" t="s">
+        <v>87</v>
+      </c>
+      <c r="C176" t="s">
+        <v>84</v>
+      </c>
+      <c r="D176" t="s">
+        <v>104</v>
+      </c>
+      <c r="E176">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A177" t="s">
+        <v>64</v>
+      </c>
+      <c r="B177" t="s">
+        <v>87</v>
+      </c>
+      <c r="C177" t="s">
+        <v>84</v>
+      </c>
+      <c r="D177" t="s">
+        <v>104</v>
+      </c>
+      <c r="E177">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A178" t="s">
+        <v>64</v>
+      </c>
+      <c r="B178" t="s">
+        <v>87</v>
+      </c>
+      <c r="C178" t="s">
+        <v>84</v>
+      </c>
+      <c r="D178" t="s">
+        <v>104</v>
+      </c>
+      <c r="E178">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A179" t="s">
+        <v>94</v>
+      </c>
+      <c r="B179" t="s">
+        <v>83</v>
+      </c>
+      <c r="C179" t="s">
+        <v>84</v>
+      </c>
+      <c r="D179" t="s">
+        <v>103</v>
+      </c>
+      <c r="E179">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A180" t="s">
+        <v>94</v>
+      </c>
+      <c r="B180" t="s">
+        <v>87</v>
+      </c>
+      <c r="C180" t="s">
+        <v>84</v>
+      </c>
+      <c r="D180" t="s">
+        <v>104</v>
+      </c>
+      <c r="E180">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A181" t="s">
+        <v>65</v>
+      </c>
+      <c r="B181" t="s">
+        <v>83</v>
+      </c>
+      <c r="C181" t="s">
+        <v>84</v>
+      </c>
+      <c r="D181" t="s">
+        <v>103</v>
+      </c>
+      <c r="E181">
+        <v>5.3333333333333337E-2</v>
+      </c>
+    </row>
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A182" t="s">
+        <v>65</v>
+      </c>
+      <c r="B182" t="s">
+        <v>87</v>
+      </c>
+      <c r="C182" t="s">
+        <v>84</v>
+      </c>
+      <c r="D182" t="s">
+        <v>104</v>
+      </c>
+      <c r="E182">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A183" t="s">
+        <v>66</v>
+      </c>
+      <c r="B183" t="s">
+        <v>83</v>
+      </c>
+      <c r="C183" t="s">
+        <v>84</v>
+      </c>
+      <c r="D183" t="s">
+        <v>103</v>
+      </c>
+      <c r="E183">
+        <v>0.41884816753926701</v>
+      </c>
+    </row>
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A184" t="s">
+        <v>66</v>
+      </c>
+      <c r="B184" t="s">
+        <v>87</v>
+      </c>
+      <c r="C184" t="s">
+        <v>84</v>
+      </c>
+      <c r="D184" t="s">
+        <v>104</v>
+      </c>
+      <c r="E184">
+        <v>1.256544502617801</v>
+      </c>
+    </row>
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A185" t="s">
+        <v>67</v>
+      </c>
+      <c r="B185" t="s">
+        <v>83</v>
+      </c>
+      <c r="C185" t="s">
+        <v>84</v>
+      </c>
+      <c r="D185" t="s">
+        <v>103</v>
+      </c>
+      <c r="E185">
+        <v>0.41884816753926701</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A186" t="s">
+        <v>67</v>
+      </c>
+      <c r="B186" t="s">
+        <v>87</v>
+      </c>
+      <c r="C186" t="s">
+        <v>84</v>
+      </c>
+      <c r="D186" t="s">
+        <v>104</v>
+      </c>
+      <c r="E186">
+        <v>1.256544502617801</v>
+      </c>
+    </row>
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A187" t="s">
+        <v>68</v>
+      </c>
+      <c r="B187" t="s">
+        <v>83</v>
+      </c>
+      <c r="C187" t="s">
+        <v>84</v>
+      </c>
+      <c r="D187" t="s">
+        <v>103</v>
+      </c>
+      <c r="E187">
+        <v>4.7999999999999996E-3</v>
+      </c>
+    </row>
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A188" t="s">
+        <v>68</v>
+      </c>
+      <c r="B188" t="s">
+        <v>87</v>
+      </c>
+      <c r="C188" t="s">
+        <v>84</v>
+      </c>
+      <c r="D188" t="s">
+        <v>104</v>
+      </c>
+      <c r="E188">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A189" t="s">
+        <v>69</v>
+      </c>
+      <c r="B189" t="s">
+        <v>83</v>
+      </c>
+      <c r="C189" t="s">
+        <v>84</v>
+      </c>
+      <c r="D189" t="s">
+        <v>103</v>
+      </c>
+      <c r="E189">
+        <v>4.7999999999999996E-3</v>
+      </c>
+    </row>
+    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A190" t="s">
+        <v>69</v>
+      </c>
+      <c r="B190" t="s">
+        <v>87</v>
+      </c>
+      <c r="C190" t="s">
+        <v>84</v>
+      </c>
+      <c r="D190" t="s">
+        <v>104</v>
+      </c>
+      <c r="E190">
+        <v>3.2000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A191" t="s">
+        <v>70</v>
+      </c>
+      <c r="B191" t="s">
+        <v>83</v>
+      </c>
+      <c r="C191" t="s">
+        <v>84</v>
+      </c>
+      <c r="D191" t="s">
+        <v>103</v>
+      </c>
+      <c r="E191">
+        <v>4.7999999999999996E-3</v>
+      </c>
+    </row>
+    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A192" t="s">
+        <v>70</v>
+      </c>
+      <c r="B192" t="s">
+        <v>87</v>
+      </c>
+      <c r="C192" t="s">
+        <v>84</v>
+      </c>
+      <c r="D192" t="s">
+        <v>104</v>
+      </c>
+      <c r="E192">
+        <v>3.2000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A193" t="s">
+        <v>71</v>
+      </c>
+      <c r="B193" t="s">
+        <v>83</v>
+      </c>
+      <c r="C193" t="s">
+        <v>84</v>
+      </c>
+      <c r="D193" t="s">
+        <v>103</v>
+      </c>
+      <c r="E193">
+        <v>2.6666666666666666E-3</v>
+      </c>
+    </row>
+    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A194" t="s">
+        <v>71</v>
+      </c>
+      <c r="B194" t="s">
+        <v>87</v>
+      </c>
+      <c r="C194" t="s">
+        <v>84</v>
+      </c>
+      <c r="D194" t="s">
+        <v>104</v>
+      </c>
+      <c r="E194">
+        <v>1.6E-2</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A195" t="s">
+        <v>95</v>
+      </c>
+      <c r="B195" t="s">
+        <v>83</v>
+      </c>
+      <c r="C195" t="s">
+        <v>84</v>
+      </c>
+      <c r="D195" t="s">
+        <v>103</v>
+      </c>
+      <c r="E195">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A196" t="s">
+        <v>95</v>
+      </c>
+      <c r="B196" t="s">
+        <v>87</v>
+      </c>
+      <c r="C196" t="s">
+        <v>84</v>
+      </c>
+      <c r="D196" t="s">
+        <v>104</v>
+      </c>
+      <c r="E196">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A197" t="s">
+        <v>96</v>
+      </c>
+      <c r="B197" t="s">
+        <v>83</v>
+      </c>
+      <c r="C197" t="s">
+        <v>84</v>
+      </c>
+      <c r="D197" t="s">
+        <v>103</v>
+      </c>
+      <c r="E197">
+        <v>0.64</v>
+      </c>
+    </row>
+    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A198" t="s">
+        <v>96</v>
+      </c>
+      <c r="B198" t="s">
+        <v>87</v>
+      </c>
+      <c r="C198" t="s">
+        <v>84</v>
+      </c>
+      <c r="D198" t="s">
+        <v>104</v>
+      </c>
+      <c r="E198">
+        <v>5.12</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A199" t="s">
+        <v>73</v>
+      </c>
+      <c r="B199" t="s">
+        <v>83</v>
+      </c>
+      <c r="C199" t="s">
+        <v>84</v>
+      </c>
+      <c r="D199" t="s">
+        <v>103</v>
+      </c>
+      <c r="E199">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A200" t="s">
+        <v>73</v>
+      </c>
+      <c r="B200" t="s">
+        <v>87</v>
+      </c>
+      <c r="C200" t="s">
+        <v>84</v>
+      </c>
+      <c r="D200" t="s">
+        <v>104</v>
+      </c>
+      <c r="E200">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A201" t="s">
+        <v>97</v>
+      </c>
+      <c r="B201" t="s">
+        <v>83</v>
+      </c>
+      <c r="C201" t="s">
+        <v>84</v>
+      </c>
+      <c r="D201" t="s">
+        <v>103</v>
+      </c>
+      <c r="E201">
+        <v>0.64</v>
+      </c>
+    </row>
+    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A202" t="s">
+        <v>97</v>
+      </c>
+      <c r="B202" t="s">
+        <v>87</v>
+      </c>
+      <c r="C202" t="s">
+        <v>84</v>
+      </c>
+      <c r="D202" t="s">
+        <v>104</v>
+      </c>
+      <c r="E202">
+        <v>3.84</v>
+      </c>
+    </row>
+    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A203" t="s">
+        <v>74</v>
+      </c>
+      <c r="B203" t="s">
+        <v>83</v>
+      </c>
+      <c r="C203" t="s">
+        <v>84</v>
+      </c>
+      <c r="D203" t="s">
+        <v>103</v>
+      </c>
+      <c r="E203">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A204" t="s">
+        <v>74</v>
+      </c>
+      <c r="B204" t="s">
+        <v>87</v>
+      </c>
+      <c r="C204" t="s">
+        <v>84</v>
+      </c>
+      <c r="D204" t="s">
+        <v>104</v>
+      </c>
+      <c r="E204">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A205" t="s">
+        <v>98</v>
+      </c>
+      <c r="B205" t="s">
+        <v>83</v>
+      </c>
+      <c r="C205" t="s">
+        <v>84</v>
+      </c>
+      <c r="D205" t="s">
+        <v>103</v>
+      </c>
+      <c r="E205">
+        <v>0.64</v>
+      </c>
+    </row>
+    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A206" t="s">
+        <v>98</v>
+      </c>
+      <c r="B206" t="s">
+        <v>87</v>
+      </c>
+      <c r="C206" t="s">
+        <v>84</v>
+      </c>
+      <c r="D206" t="s">
+        <v>104</v>
+      </c>
+      <c r="E206">
+        <v>4.4800000000000004</v>
+      </c>
+    </row>
+    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A207" t="s">
+        <v>99</v>
+      </c>
+      <c r="B207" t="s">
+        <v>83</v>
+      </c>
+      <c r="C207" t="s">
+        <v>84</v>
+      </c>
+      <c r="D207" t="s">
+        <v>103</v>
+      </c>
+      <c r="E207">
+        <v>1.28</v>
+      </c>
+    </row>
+    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A208" t="s">
+        <v>99</v>
+      </c>
+      <c r="B208" t="s">
+        <v>87</v>
+      </c>
+      <c r="C208" t="s">
+        <v>84</v>
+      </c>
+      <c r="D208" t="s">
+        <v>104</v>
+      </c>
+      <c r="E208">
+        <v>7.68</v>
+      </c>
+    </row>
+    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A209" t="s">
+        <v>75</v>
+      </c>
+      <c r="B209" t="s">
+        <v>83</v>
+      </c>
+      <c r="C209" t="s">
+        <v>84</v>
+      </c>
+      <c r="D209" t="s">
+        <v>103</v>
+      </c>
+      <c r="E209">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A210" t="s">
+        <v>75</v>
+      </c>
+      <c r="B210" t="s">
+        <v>87</v>
+      </c>
+      <c r="C210" t="s">
+        <v>84</v>
+      </c>
+      <c r="D210" t="s">
+        <v>104</v>
+      </c>
+      <c r="E210">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A211" t="s">
+        <v>100</v>
+      </c>
+      <c r="B211" t="s">
+        <v>83</v>
+      </c>
+      <c r="C211" t="s">
+        <v>84</v>
+      </c>
+      <c r="D211" t="s">
+        <v>103</v>
+      </c>
+      <c r="E211">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A212" t="s">
+        <v>100</v>
+      </c>
+      <c r="B212" t="s">
+        <v>87</v>
+      </c>
+      <c r="C212" t="s">
+        <v>84</v>
+      </c>
+      <c r="D212" t="s">
+        <v>104</v>
+      </c>
+      <c r="E212">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A213" t="s">
+        <v>101</v>
+      </c>
+      <c r="B213" t="s">
+        <v>83</v>
+      </c>
+      <c r="C213" t="s">
+        <v>84</v>
+      </c>
+      <c r="D213" t="s">
+        <v>103</v>
+      </c>
+      <c r="E213">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A214" t="s">
+        <v>101</v>
+      </c>
+      <c r="B214" t="s">
+        <v>87</v>
+      </c>
+      <c r="C214" t="s">
+        <v>84</v>
+      </c>
+      <c r="D214" t="s">
+        <v>104</v>
+      </c>
+      <c r="E214">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A215" t="s">
+        <v>76</v>
+      </c>
+      <c r="B215" t="s">
+        <v>83</v>
+      </c>
+      <c r="C215" t="s">
+        <v>84</v>
+      </c>
+      <c r="D215" t="s">
+        <v>103</v>
+      </c>
+      <c r="E215">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A216" t="s">
+        <v>76</v>
+      </c>
+      <c r="B216" t="s">
+        <v>87</v>
+      </c>
+      <c r="C216" t="s">
+        <v>84</v>
+      </c>
+      <c r="D216" t="s">
+        <v>104</v>
+      </c>
+      <c r="E216">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A217" t="s">
+        <v>77</v>
+      </c>
+      <c r="B217" t="s">
+        <v>83</v>
+      </c>
+      <c r="C217" t="s">
+        <v>84</v>
+      </c>
+      <c r="D217" t="s">
+        <v>103</v>
+      </c>
+      <c r="E217">
+        <v>11.2</v>
+      </c>
+    </row>
+    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A218" t="s">
+        <v>77</v>
+      </c>
+      <c r="B218" t="s">
+        <v>87</v>
+      </c>
+      <c r="C218" t="s">
+        <v>84</v>
+      </c>
+      <c r="D218" t="s">
+        <v>104</v>
+      </c>
+      <c r="E218">
+        <v>27.2</v>
+      </c>
+    </row>
+    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A219" t="s">
+        <v>80</v>
+      </c>
+      <c r="B219" t="s">
+        <v>83</v>
+      </c>
+      <c r="C219" t="s">
+        <v>84</v>
+      </c>
+      <c r="D219" t="s">
+        <v>103</v>
+      </c>
+      <c r="E219">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A220" t="s">
+        <v>80</v>
+      </c>
+      <c r="B220" t="s">
+        <v>87</v>
+      </c>
+      <c r="C220" t="s">
+        <v>84</v>
+      </c>
+      <c r="D220" t="s">
+        <v>104</v>
+      </c>
+      <c r="E220">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A221" t="s">
+        <v>102</v>
+      </c>
+      <c r="B221" t="s">
+        <v>83</v>
+      </c>
+      <c r="C221" t="s">
+        <v>84</v>
+      </c>
+      <c r="D221" t="s">
+        <v>103</v>
+      </c>
+      <c r="E221">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A222" t="s">
+        <v>102</v>
+      </c>
+      <c r="B222" t="s">
+        <v>87</v>
+      </c>
+      <c r="C222" t="s">
+        <v>84</v>
+      </c>
+      <c r="D222" t="s">
+        <v>104</v>
+      </c>
+      <c r="E222">
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>